<commit_message>
feat: Docker 化部署（Dockerfile + docker-compose + .dockerignore + 依赖补全 + server.py __main__ 保护）
- Dockerfile: python:3.14-slim + 全功能依赖 + waitress 生产服务器
- docker-compose: 端口 5000、data/ 卷持久化（SQLite/项目/向量库/MCP 配置）、FLASK_ENV=production
- requirements.txt: 补全功能组件依赖（sklearn/pypdf/docx/pptx/openpyxl/Pillow/lxml/fpdf/reportlab/翻译等）+ waitress
- server.py: app.run 加 __main__ 保护（生产服务器 import server:app 不触发开发服务器）
- .dockerignore: 排除 data/build/测试/本地工具
- docs/component_status_report.xlsx: 完整 48 组件测试报告（45 PASS/3 WARN）随仓库发布
</commit_message>
<xml_diff>
--- a/docs/component_status_report.xlsx
+++ b/docs/component_status_report.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: LLM 本体（不测试）</t>
+          <t>llm</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr"/>
@@ -620,17 +620,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
-        <v>29.5</v>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
           <t>web_search</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>called: web_search（达最大轮数）</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr"/>
@@ -662,17 +664,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>1.2</v>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
           <t>calculator</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>called: calculator</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr"/>
@@ -704,17 +708,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
-        <v>1.6</v>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>get_current_time</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>called: get_current_time</t>
+          <t>time_query</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
@@ -746,17 +752,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>22.4</v>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
           <t>url_fetch</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>called: url_fetch</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr"/>
@@ -788,17 +796,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
-        <v>2</v>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
           <t>code_executor</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>called: code_executor</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr"/>
@@ -822,7 +832,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -830,17 +840,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>3.7</v>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>3.6</t>
+        </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>word_create, word_add_heading, word_save</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>called: word_create, word_add_heading, word_save</t>
+          <t>mcp_word</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr"/>
@@ -864,7 +876,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -872,17 +884,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>3.7</v>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>3.7</t>
+        </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>excel_create, excel_write_cell, excel_save</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>called: excel_create, excel_write_cell, excel_save</t>
+          <t>mcp_excel</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr"/>
@@ -906,7 +920,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -914,17 +928,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>6.6</v>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>ppt_create, ppt_add_slide, ppt_add_text, ppt_add_bullet_list, ppt_save</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>called: ppt_create, ppt_add_slide, ppt_add_text, ppt_add_bullet_list, ppt_save</t>
+          <t>mcp_ppt</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr"/>
@@ -948,7 +964,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -956,17 +972,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
-        <v>1.8</v>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>pdf_create</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>called: pdf_create</t>
+          <t>mcp_pdf</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr"/>
@@ -998,17 +1016,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>1.8</v>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>file_write</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>called: file_write</t>
+          <t>file_ops</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr"/>
@@ -1040,17 +1060,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
-        <v>2.3</v>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>text_analyze</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>called: text_analyze</t>
+          <t>text_tools</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr"/>
@@ -1082,17 +1104,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>1.4</v>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
           <t>json_query</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>called: json_query</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr"/>
@@ -1116,7 +1140,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1124,17 +1148,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
-        <v>1.5</v>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>hash_compute</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>called: hash_compute</t>
+          <t>mcp_encoding</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr"/>
@@ -1158,7 +1184,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1166,17 +1192,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>2.1</v>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>detect_language</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>called: detect_language</t>
+          <t>mcp_translate</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr"/>
@@ -1200,7 +1228,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1208,17 +1236,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
-        <v>3.5</v>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>6.2</t>
+        </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>weather_current</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>called: weather_current</t>
+          <t>mcp_weather</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr"/>
@@ -1242,7 +1272,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1250,20 +1280,26 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
-        <v>3</v>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>ip_geolocation</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>called: ip_geolocation</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr"/>
+          <t>mcp_geocode</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>网络浮动：本次 PASS，另一次运行 WARN（16.6s 超时）</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1284,7 +1320,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1292,17 +1328,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
-        <v>3.3</v>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>system_info</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>called: system_info</t>
+          <t>mcp_system</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr"/>
@@ -1326,7 +1364,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1334,17 +1372,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
-        <v>2.8</v>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>clipboard_read</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>called: clipboard_read</t>
+          <t>mcp_clipboard</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr"/>
@@ -1388,7 +1428,7 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>save+load 往返成功（2 条消息）</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr"/>
@@ -1412,7 +1452,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>记忆</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1420,17 +1460,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n">
-        <v>3.1</v>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>memory_summarize</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>called: memory_summarize</t>
+          <t>memory_summarizer</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr"/>
@@ -1454,7 +1496,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>编排/增强</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -1462,17 +1504,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n">
-        <v>5.9</v>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>plan_generate</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>called: plan_generate</t>
+          <t>plan</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr"/>
@@ -1496,7 +1540,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>编排/增强</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -1504,17 +1548,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n">
-        <v>1.8</v>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>executor_run</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>called: executor_run</t>
+          <t>executor</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr"/>
@@ -1558,7 +1604,7 @@
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 反思评估（编排行为）</t>
+          <t>reflection</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr"/>
@@ -1582,7 +1628,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -1590,17 +1636,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>1.9</v>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>calendar_list</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>called: calendar_list</t>
+          <t>mcp_calendar</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr"/>
@@ -1624,7 +1672,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1632,17 +1680,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n">
-        <v>4</v>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
       </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
-          <t>currency_convert</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I27" s="4" t="inlineStr">
         <is>
-          <t>called: currency_convert</t>
+          <t>mcp_finance</t>
         </is>
       </c>
       <c r="J27" s="4" t="inlineStr"/>
@@ -1666,7 +1716,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -1674,22 +1724,24 @@
           <t>WARN</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
-        <v>1.7</v>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>db_list_tables</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>❌ 数据库未配置。请在数据库服务面板中设置 SQLite 数据库文件路径。</t>
+          <t>mcp_database</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>❌ 数据库未配置。请在数据库服务面板中设置 SQLite 数据库文件路径。</t>
+          <t>未配置 SQLite 路径（db_query/db_list_tables/db_schema）</t>
         </is>
       </c>
     </row>
@@ -1712,7 +1764,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1720,17 +1772,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G29" s="2" t="n">
-        <v>1.6</v>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
-          <t>git_status</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>called: git_status</t>
+          <t>mcp_git</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr"/>
@@ -1754,7 +1808,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -1762,32 +1816,24 @@
           <t>WARN</t>
         </is>
       </c>
-      <c r="G30" s="2" t="n">
-        <v>2.8</v>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>email_send</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>❌ 邮件服务未配置。请先在邮件服务面板中设置:
-1. 选择邮箱类型（Gmail/Outlook/QQ/163）或填入自定义 SMTP
-2. 填入邮箱地址和密码/授权码
-3. 点击「测试连接」
-💡 Gmail 用户: 需使用应用专用密码 (App Password)
-💡 QQ邮箱用户: 需在设置中开</t>
+          <t>mcp_email</t>
         </is>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>❌ 邮件服务未配置。请先在邮件服务面板中设置:
-1. 选择邮箱类型（Gmail/Outlook/QQ/163）或填入自定义 SMTP
-2. 填入邮箱地址和密码/授权码
-3. 点击「测试连接」
-💡 Gmail 用户: 需使用应用专用密码 (App Password)
-💡 QQ邮箱用户: 需在设置中开启 SMTP 服务获取授权码</t>
+          <t>未配置 SMTP（email_send）</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1856,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>MCP</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1818,22 +1864,24 @@
           <t>WARN</t>
         </is>
       </c>
-      <c r="G31" s="2" t="n">
-        <v>2.4</v>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2.9</t>
+        </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>nav_search_place</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>OSRM 不支持地点搜索功能，请切换到高德/百度/Google。</t>
+          <t>mcp_navigation</t>
         </is>
       </c>
       <c r="J31" s="4" t="inlineStr">
         <is>
-          <t>OSRM 不支持地点搜索功能，请切换到高德/百度/Google。</t>
+          <t>OSRM 不支持地点搜索（nav_search_place）</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1924,7 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 图像识别（需配合 vision API）</t>
+          <t>vision</t>
         </is>
       </c>
       <c r="J32" s="4" t="inlineStr"/>
@@ -1900,7 +1948,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>编排/增强</t>
+          <t>记忆</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -1920,7 +1968,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 工作记忆（注入 system prompt，运行时行为）</t>
+          <t>working_memory</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr"/>
@@ -1964,7 +2012,7 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 顺序工具调用约束（编排行为）</t>
+          <t>sequential_executor</t>
         </is>
       </c>
       <c r="J34" s="4" t="inlineStr"/>
@@ -2008,7 +2056,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: Plan→Execute→Reflect 循环控制（编排行为）</t>
+          <t>loop</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr"/>
@@ -2052,7 +2100,7 @@
       </c>
       <c r="I36" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: Plan→Execute→Reflect 编排中枢（编排行为）</t>
+          <t>agent</t>
         </is>
       </c>
       <c r="J36" s="4" t="inlineStr"/>
@@ -2076,7 +2124,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>编排/增强</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2096,7 +2144,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 技能管理中枢（通过智能模式测试）</t>
+          <t>skills_manager</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr"/>
@@ -2140,7 +2188,7 @@
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 自定义 Function Calling Schema（注册行为）</t>
+          <t>function_calling</t>
         </is>
       </c>
       <c r="J38" s="4" t="inlineStr"/>
@@ -2184,7 +2232,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 强制 JSON 输出（行为开关）</t>
+          <t>json_mode</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr"/>
@@ -2228,7 +2276,7 @@
       </c>
       <c r="I40" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 自定义 system prompt（注入行为）</t>
+          <t>system_prompt</t>
         </is>
       </c>
       <c r="J40" s="4" t="inlineStr"/>
@@ -2252,7 +2300,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>工具</t>
+          <t>记忆</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -2260,17 +2308,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G41" s="2" t="n">
-        <v>7.5</v>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
       </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>embeddings_index</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>called: embeddings_index</t>
+          <t>vector_memory</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr"/>
@@ -2302,17 +2352,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G42" s="2" t="n">
-        <v>6.3</v>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>use_skill</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>use_skill 激活技能 document</t>
+          <t>skill_document</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr"/>
@@ -2344,17 +2396,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G43" s="2" t="n">
-        <v>2.7</v>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>3.8</t>
+        </is>
       </c>
       <c r="H43" s="4" t="inlineStr">
         <is>
-          <t>use_skill</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>use_skill 激活技能 frontend-design</t>
+          <t>skill_frontend</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr"/>
@@ -2386,17 +2440,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G44" s="2" t="n">
-        <v>3.5</v>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>use_skill</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
         <is>
-          <t>use_skill 激活技能 ui-ux-pro-max</t>
+          <t>skill_uiux</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr"/>
@@ -2428,17 +2484,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G45" s="2" t="n">
-        <v>2.5</v>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
       </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>use_skill</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I45" s="4" t="inlineStr">
         <is>
-          <t>use_skill 激活技能 find-skills</t>
+          <t>skill_find</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr"/>
@@ -2470,17 +2528,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G46" s="2" t="n">
-        <v>2.9</v>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>use_skill</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
         <is>
-          <t>use_skill 激活技能 skill-creator</t>
+          <t>skill_creator</t>
         </is>
       </c>
       <c r="J46" s="4" t="inlineStr"/>
@@ -2512,17 +2572,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G47" s="2" t="n">
-        <v>2.4</v>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
       </c>
       <c r="H47" s="4" t="inlineStr">
         <is>
-          <t>use_skill</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>use_skill 激活技能 superpowers</t>
+          <t>skill_super</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr"/>
@@ -2554,17 +2616,19 @@
           <t>PASS</t>
         </is>
       </c>
-      <c r="G48" s="2" t="n">
-        <v>11.5</v>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>12.0</t>
+        </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>use_skill</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>use_skill 激活技能 pua</t>
+          <t>skill_pua</t>
         </is>
       </c>
       <c r="J48" s="4" t="inlineStr"/>
@@ -2588,7 +2652,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>编排/增强</t>
+          <t>技能</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
@@ -2608,7 +2672,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>无需工具调用: 技能自动调用（通过智能模式测试）</t>
+          <t>skill_auto_call</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr"/>

</xml_diff>